<commit_message>
Update Margin Bridge with channel-mix and portfolio tier-mix sizing
Adds two newly-sized levers: channel mix shift (Wholesale -> DTC,
+1.36pt grounded to the approved Item 4 store plan, up to +4.47pt
under an aggressive scenario) and portfolio tier-mix optimization
(+1.65pt moderate, replacing the old floor-fix-only figure, up to
+5.49pt theoretical ceiling). Updates the headline reconciliation:
quantified upside rises from ~2.8pt to ~5.1pt, residual narrows from
~10.5-11.5pt to ~9.2pt (64% of the +14.3pt target) -- still the
majority of the gap, but real progress.
</commit_message>
<xml_diff>
--- a/workshop_prep/bob_marginbridge_backup.xlsx
+++ b/workshop_prep/bob_marginbridge_backup.xlsx
@@ -10,8 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lever Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix - Current" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix - Sensitivity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Tier-Mix Scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -457,7 +460,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The headline reconciliation: target +14.3pt vs. what has actually been quantified across Items 1-6, and the residual</t>
+          <t>UPDATED headline reconciliation: target +14.3pt vs. what has actually been quantified across Items 1-6 plus the channel-mix and tier-mix sizing added this round, and the residual</t>
         </is>
       </c>
     </row>
@@ -476,22 +479,58 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Basis Mismatch Check</t>
+          <t>Channel Mix - Current</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+          <t>2025 sales, GM% and share by Sales Channel (Wholesale/Retail/E-com/Marketplace) -- the base data for the channel-mix sizing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Channel Mix - Sensitivity</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sensitivity table: blended company GM% at different Wholesale-share levels, holding each channel's own 2025 margin rate fixed, plus the concrete scenario anchored to the Item 4 new-store plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Portfolio Tier-Mix Scenarios</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Three tier-mix scenarios (floor-fix / Workhorse-level turnaround / theoretical Hero-level ceiling) for Problem Child and Thin tiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Basis Mismatch Check</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Special-Acct Mix Decomposition</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Fresh Laspeyres mix/rate decomposition of the Core vs Special-account (XXL/Zalando/China/Stadium) blended margin, FY2024-&gt;FY2025</t>
         </is>
@@ -508,12 +547,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,11 +565,6 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -544,94 +577,88 @@
           <t>39.2% -&gt; 53.5% (+14.3pt)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>MTP target, established at engagement start</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Quantified upside, conservative reading (avoids double-counting FW27 gap vs general price-erosion)</t>
+          <t>General mix-adjusted price erosion (Item 2), if reversed</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>~2.8pt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Sum of: general price erosion (1.89pt) + Problem Child pricing fix (0.69pt) + Reorder margin gap (0.19pt)</t>
+          <t>+1.89pt</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quantified upside, generous reading (uses FW27 gap instead of general erosion line)</t>
+          <t>Portfolio tier-mix, moderate scenario (PC + Thin to Workhorse-level)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>~3.8pt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sum of: FW27 Wholesale gap (2.92pt) + Problem Child pricing fix (0.69pt) + Reorder margin gap (0.19pt)</t>
+          <t>+1.65pt</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RESIDUAL -- unexplained by anything sized in Items 1-6</t>
+          <t>Wholesale Reorder margin gap (Item 5), if closed</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>~10.5 to 11.5pt (73-80% of the total target gap)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>This note</t>
+          <t>+0.19pt</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Known negative drags during the bridge period (not netted into the above)</t>
+          <t>Channel mix shift, grounded to the approved Item 4 store plan</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Special-account mix -0.43pt (FY24-&gt;25 actual, may continue); New-store start-up losses (EBIT, unsized in GM terms)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>This note; Item 4</t>
+          <t>+1.36pt</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Basis mismatch at the FY2025A starting point itself</t>
+          <t>UPDATED quantified total (grounded/moderate reading)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sales-extract blended margin 41.0% vs. P&amp;L Gross Margin 39.2% -- 1.8pt unreconciled</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>This note</t>
+          <t>~5.1pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>UPDATED RESIDUAL -- still unexplained</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>~9.2pt (64% of target)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Outer-bound context (not additive, alternative aggressive scenarios)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Channel mix at WS=50%: +4.47pt ceiling. Entire portfolio at Hero-level: +5.49pt ceiling.</t>
         </is>
       </c>
     </row>
@@ -911,6 +938,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sales_2025</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>GM_2025</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Share_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>658416100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.365913</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.751</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>123001900</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.489854</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E-com</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>94129810</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.612406</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1605617</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.714351</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>WS_share_pct</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Blended_GM_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Change_pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="B2" t="n">
+        <v>41.03</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>70</v>
+      </c>
+      <c r="B3" t="n">
+        <v>41.94</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B4" t="n">
+        <v>42.83</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B5" t="n">
+        <v>43.72</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B6" t="n">
+        <v>44.62</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B7" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SEK_impact_M</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Pt_of_company_sales</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A: Problem Child (Core Pricing Fix, 88.5M) -&gt; 40% GM floor</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Conservative -- floor only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B1: Problem Child (88.5M) -&gt; Workhorse-level margin (47.5%)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Moderate -- genuine turnaround, not just floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B2: Thin tier (8.1M) replaced at Workhorse-level margin (47.5%)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Moderate -- assumes exited volume replaced by equivalent-value product, not just deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B total (B1+B2) -- recommended working assumption</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>13.97</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Supersedes Scenario A as the working number</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C: ENTIRE core portfolio (649.8M) -&gt; Hero-level margin (53.5%)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Theoretical ceiling only -- not a real plan (would require all 1,860 franchises, incl. Harvest/Thin/Exited, to perform like the best 34)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1007,7 +1374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add base-year normalization investigation to the Margin Bridge
Tests whether FY2025A was artificially depressed by one-off COVID-era
inventory clearance -- finds the opposite for the smaller COGS
provision/defectives lines (2024 was worse there, already reflected
in the FY25A base), but surfaces a real, previously-unexamined finding:
Direct Cost of Sales ratio spiked specifically in FY2025 (-3.5pt vs
FY2024A), and YTD2026 data shows it already reversing sharply
(-5.1pt vs the same period last year, Gross Margin +2.5pt). Flagged
as a strong signal worth 2.5-5pt but deliberately not added to the
quantified total pending disentanglement from the XXL mix effect,
which requires 2026 article-level data not available in this
engagement.
</commit_message>
<xml_diff>
--- a/workshop_prep/bob_marginbridge_backup.xlsx
+++ b/workshop_prep/bob_marginbridge_backup.xlsx
@@ -13,8 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix - Current" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix - Sensitivity" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Tier-Mix Scenarios" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base-Year Normalization" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base-Year Findings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -515,25 +517,173 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Basis Mismatch Check</t>
+          <t>Base-Year Normalization</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+          <t>Direct Cost of Sales ratio and 'other COGS lines' (Defectives/Inventory Provision/FX Difference/Other) as % of Net Sales, FY2024A/FY2025A/YTD2025/YTD2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Base-Year Findings</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>The four specific findings from the base-year investigation, with read/interpretation for each</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Basis Mismatch Check</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Special-Acct Mix Decomposition</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Fresh Laspeyres mix/rate decomposition of the Core vs Special-account (XXL/Zalando/China/Stadium) blended margin, FY2024-&gt;FY2025</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>GM%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C2" t="n">
+        <v>619614344.6793205</v>
+      </c>
+      <c r="D2" t="n">
+        <v>283394704.7593222</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.4573727306232594</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C3" t="n">
+        <v>649760107.9369266</v>
+      </c>
+      <c r="D3" t="n">
+        <v>301131325.6574844</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.4634500055930115</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C4" t="n">
+        <v>163622850.9118249</v>
+      </c>
+      <c r="D4" t="n">
+        <v>60866600.45182489</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3719932766886297</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C5" t="n">
+        <v>227393297.1590489</v>
+      </c>
+      <c r="D5" t="n">
+        <v>58837518.77904887</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.258747814971412</v>
       </c>
     </row>
   </sheetData>
@@ -1278,95 +1428,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Net_Sales_KSEK</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>DirectCOGS_pct_of_sales</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>OtherProvisionLines_pct_of_sales</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Gross_Margin_pct</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P&amp;L Gross Margin, FY2025A (bob_financialdata_2025.xlsx)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>39.2%</t>
-        </is>
+          <t>FY2024A (full year)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>736987</v>
+      </c>
+      <c r="C2" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P&amp;L Net Sales, FY2025A</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>846,293,000 SEK</t>
-        </is>
+          <t>FY2025A (full year)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>846293</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="E3" t="n">
+        <v>39.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P&amp;L Gross Profit, FY2025A</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>331,435,000 SEK</t>
-        </is>
+          <t>YTD 2025 (comparative, same period as YTD26)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>371056</v>
+      </c>
+      <c r="C4" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E4" t="n">
+        <v>39.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sales-extract blended margin (Garp SEK Margin / Garp SEK Sales), FY2025, all channels+accounts</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>41.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1.8pt -- not reconciled in this engagement</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Plausible causes (not verified)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Different cost inclusions (e.g. logistics/freight allocated in P&amp;L COGS but not in Garp COGS), different revenue scope (Garp extract may exclude some entities/adjustments the P&amp;L includes), or a timing/consolidation difference</t>
-        </is>
+          <t>YTD 2026 (current)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>294713</v>
+      </c>
+      <c r="C5" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>41.7</v>
       </c>
     </row>
   </sheetData>
@@ -1380,117 +1552,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Finding</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>GM%</t>
+          <t>Read</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C2" t="n">
-        <v>619614344.6793205</v>
-      </c>
-      <c r="D2" t="n">
-        <v>283394704.7593222</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.4573727306232594</v>
+          <t>Other/Provision/Defectives/FX-difference COGS lines, swing FY2024-&gt;FY2025</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>+52.5M SEK = +6.2pt of company sales</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ALREADY REALIZED within the FY2025A base -- 2024 had the heavier one-off charges (Other COS -30.0M, Defectives -7.1M, Inventory Provision -5.7M charge, Other COS2 -15.1M), not 2025. This means FY2025A is NOT artificially depressed by one-off inventory charges relative to 2024 -- if anything it already reflects an improvement. The original 'is 2025 a depressed base year' hypothesis is NOT supported on this specific decomposition.</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C3" t="n">
-        <v>649760107.9369266</v>
-      </c>
-      <c r="D3" t="n">
-        <v>301131325.6574844</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.4634500055930115</v>
+          <t>Direct Cost of Sales ratio, FY2024A -&gt; FY2025A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>56.9% -&gt; 60.4% of Net Sales = -3.5pt deterioration</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A genuine, real, unexplained swing in the main COGS line specifically in FY2025 -- this is the company-wide P&amp;L confirmation of the per-unit COGS increases already found in Item 2 (Wholesale Reorder COGS/unit +12-44%, Retail COGS/unit +13.6%), attributed to FX per CEO direction but never verified against transaction-level data.</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C4" t="n">
-        <v>163622850.9118249</v>
-      </c>
-      <c r="D4" t="n">
-        <v>60866600.45182489</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.3719932766886297</v>
+          <t>Direct Cost of Sales ratio, YTD2025 (comparative) -&gt; YTD2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>61.2% -&gt; 56.1% = -5.1pt improvement, apples-to-apples same period</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ALREADY HAPPENING in the most current data available. This is a like-for-like YTD comparison, not full-year-vs-partial-year.</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C5" t="n">
-        <v>227393297.1590489</v>
-      </c>
-      <c r="D5" t="n">
-        <v>58837518.77904887</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.258747814971412</v>
+          <t>Gross Margin, YTD2025 (comparative) -&gt; YTD2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>39.2% -&gt; 41.7% = +2.5pt, apples-to-apples same period</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Directionally very encouraging -- current-year momentum already exceeds the FY2025A base. NOT added to the quantified running total: likely entangled with the XXL mix collapse (Item 5: XXL Wholesale sell-in -100% in Q2 2026) rather than being purely a cost-structure improvement, and cannot be disentangled without 2026 article/account-level data, which does not exist in the files provided.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P&amp;L Gross Margin, FY2025A (bob_financialdata_2025.xlsx)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>39.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P&amp;L Net Sales, FY2025A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>846,293,000 SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P&amp;L Gross Profit, FY2025A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>331,435,000 SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sales-extract blended margin (Garp SEK Margin / Garp SEK Sales), FY2025, all channels+accounts</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>41.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.8pt -- not reconciled in this engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Plausible causes (not verified)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Different cost inclusions (e.g. logistics/freight allocated in P&amp;L COGS but not in Garp COGS), different revenue scope (Garp extract may exclude some entities/adjustments the P&amp;L includes), or a timing/consolidation difference</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add competitive benchmark section to the Margin Bridge
New Section 7: five public/disclosed competitor margin comparables
(Fenix Outdoor/Fjallraven 59.4% GM, Amer Sports/Arc'teryx 57.7% GM +
21.6% op margin, VF Corp 53.5% GM, Columbia ~50-51.6% GM, Norrona 7.3%
net margin) against Haglofs' 39.2% GM / -3.5% EBIT. All five sit above
Haglofs' current margin; two sit above Haglofs' own 53.5% target.
Confirms the DTC-mix and discount-discipline levers already in this
bridge, and surfaces one new angle -- wholesale distribution curation
-- not yet analyzed anywhere in this engagement. Also names the honest
VF Corp tradeoff (margin recovery required accepting real revenue
decline) as a strategic question for the CEO/PE ownership.
</commit_message>
<xml_diff>
--- a/workshop_prep/bob_marginbridge_backup.xlsx
+++ b/workshop_prep/bob_marginbridge_backup.xlsx
@@ -15,8 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Tier-Mix Scenarios" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base-Year Normalization" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base-Year Findings" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitive Benchmark" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Mismatch Check" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special-Acct Mix Decomposition" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -541,22 +542,34 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Basis Mismatch Check</t>
+          <t>Competitive Benchmark</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+          <t>Five public/disclosed competitor gross-margin and operating/net-margin figures (Fenix Outdoor/Fjallraven, Amer Sports/Arc'teryx, VF Corp, Columbia Sportswear, Norrona) vs. Haglofs, with how each achieves it</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Basis Mismatch Check</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The 1.8pt gap between the sales-extract blended margin (41.0%) and the P&amp;L Gross Margin (39.2%) for the same FY2025A year -- unexplained by this engagement so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Special-Acct Mix Decomposition</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Fresh Laspeyres mix/rate decomposition of the Core vs Special-account (XXL/Zalando/China/Stadium) blended margin, FY2024-&gt;FY2025</t>
         </is>
@@ -568,6 +581,108 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P&amp;L Gross Margin, FY2025A (bob_financialdata_2025.xlsx)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>39.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P&amp;L Net Sales, FY2025A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>846,293,000 SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P&amp;L Gross Profit, FY2025A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>331,435,000 SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sales-extract blended margin (Garp SEK Margin / Garp SEK Sales), FY2025, all channels+accounts</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>41.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.8pt -- not reconciled in this engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Plausible causes (not verified)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Different cost inclusions (e.g. logistics/freight allocated in P&amp;L COGS but not in Garp COGS), different revenue scope (Garp extract may exclude some entities/adjustments the P&amp;L includes), or a timing/consolidation difference</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1656,94 +1771,166 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Gross_Margin</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Operating_or_Net_Margin</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>How_they_get_there</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P&amp;L Gross Margin, FY2025A (bob_financialdata_2025.xlsx)</t>
+          <t>Fenix Outdoor (Fjallraven parent)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>59.4%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1.1% EBIT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Explicitly credits margin gain to 'more direct to consumer sales and less discounting'</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P&amp;L Net Sales, FY2025A</t>
+          <t>Amer Sports (Arc'teryx parent)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>846,293,000 SEK</t>
+          <t>57.7% company-wide</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>21.6% operating margin (Technical Apparel/Arc'teryx segment)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>~60% DTC mix; curated wholesale (REI/Backcountry only); minimal discount-led marketing; ~$1,928 revenue/sqft across 160+ owned stores</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P&amp;L Gross Profit, FY2025A</t>
+          <t>VF Corp (North Face/Vans)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>331,435,000 SEK</t>
+          <t>53.5%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>n/a disclosed here</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+550bps in FY25 via a 'transformation strategy' -- cost reduction plus deliberately cutting unprofitable distribution channels (60% of Vans' revenue decline was attributed to this)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sales-extract blended margin (Garp SEK Margin / Garp SEK Sales), FY2025, all channels+accounts</t>
+          <t>Columbia Sportswear</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>41.0%</t>
+          <t>~50-51.6%</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>n/a disclosed here</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mainstream, wholesale-heavy positioning -- closest comparable to Haglofs' current channel mix, still ~11-12pt above Haglofs</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Norrona (private, Norwegian family-owned)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.8pt -- not reconciled in this engagement</t>
+          <t>not disclosed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7.3% net margin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Closest structural peer to Haglofs (small, Nordic, heritage, family-owned) -- proof the constraint isn't company size or ownership structure</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Plausible causes (not verified)</t>
+          <t>Haglofs (current, FY2025A)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Different cost inclusions (e.g. logistics/freight allocated in P&amp;L COGS but not in Garp COGS), different revenue scope (Garp extract may exclude some entities/adjustments the P&amp;L includes), or a timing/consolidation difference</t>
+          <t>39.2%</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-3.5% EBIT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>This engagement's own finding</t>
         </is>
       </c>
     </row>

</xml_diff>